<commit_message>
Refine design: home dividers, title sections, article byline, sidebar layout
- Home sections follow the source separators; new divider section style
- Breadcrumb- and title-only sections sit flush against the next section
- Article author byline as a styled section with social icon buttons
- Shared content + sidebar grid for FAQ help and article sidebars

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-adventures-2.report.xlsx
+++ b/tools/importer/reports/import-adventures-2.report.xlsx
@@ -52,7 +52,7 @@
     <t>home</t>
   </si>
   <si>
-    <t>2026-10-05T12:40:53.976Z</t>
+    <t>2026-10-05T12:57:14.334Z</t>
   </si>
   <si>
     <t>WKND Adventures and Travel</t>
@@ -73,7 +73,7 @@
     <t>about-us</t>
   </si>
   <si>
-    <t>2026-10-05T10:59:09.979Z</t>
+    <t>2026-10-05T12:44:05.176Z</t>
   </si>
   <si>
     <t>About Us</t>
@@ -94,7 +94,7 @@
     <t>adventures-2</t>
   </si>
   <si>
-    <t>2026-10-05T12:43:05.555Z</t>
+    <t>2026-10-05T12:58:44.447Z</t>
   </si>
   <si>
     <t>Adventures</t>
@@ -115,7 +115,7 @@
     <t>faqs</t>
   </si>
   <si>
-    <t>2026-10-05T10:59:21.715Z</t>
+    <t>2026-10-05T12:46:09.554Z</t>
   </si>
   <si>
     <t>FAQs</t>
@@ -136,7 +136,7 @@
     <t>magazine-landing</t>
   </si>
   <si>
-    <t>2026-10-05T12:38:13.606Z</t>
+    <t>2026-10-05T12:43:48.893Z</t>
   </si>
   <si>
     <t>Magazine</t>
@@ -403,7 +403,7 @@
     <t>magazine</t>
   </si>
   <si>
-    <t>2026-10-05T12:30:47.330Z</t>
+    <t>2026-10-05T12:52:37.973Z</t>
   </si>
   <si>
     <t>Arctic Surfing</t>
@@ -418,7 +418,7 @@
     <t>us/en/magazine/guide-la-skateparks</t>
   </si>
   <si>
-    <t>2026-10-05T12:30:51.442Z</t>
+    <t>2026-10-05T12:52:43.217Z</t>
   </si>
   <si>
     <t>Ultimate Guide to LA Skateparks</t>
@@ -433,7 +433,7 @@
     <t>us/en/magazine/san-diego-surf</t>
   </si>
   <si>
-    <t>2026-10-05T12:30:56.037Z</t>
+    <t>2026-10-05T12:52:47.898Z</t>
   </si>
   <si>
     <t>San Diego Surf Spots</t>
@@ -448,7 +448,7 @@
     <t>us/en/magazine/ski-touring</t>
   </si>
   <si>
-    <t>2026-10-05T12:31:01.328Z</t>
+    <t>2026-10-05T12:52:53.885Z</t>
   </si>
   <si>
     <t>Ski Touring</t>
@@ -463,7 +463,7 @@
     <t>us/en/magazine/western-australia</t>
   </si>
   <si>
-    <t>2026-10-05T12:31:07.855Z</t>
+    <t>2026-10-05T12:52:59.800Z</t>
   </si>
   <si>
     <t>Western Australia</t>

</xml_diff>